<commit_message>
live update 01:13:51 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -17,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -32,12 +34,30 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,10 +72,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -448,10 +474,10 @@
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="27" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="11" customWidth="1" min="30" max="30"/>
   </cols>
@@ -713,6 +739,560 @@
         </is>
       </c>
       <c r="AD2" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>01:09:20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.3984</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.4417</v>
+      </c>
+      <c r="J3" t="n">
+        <v>11000</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V3" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>0.03827989399433132</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>-0.3684402120113373</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>01:10:54</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.3984</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.4417</v>
+      </c>
+      <c r="J4" t="n">
+        <v>11000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V4" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>0.03827989399433132</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>-0.3684402120113373</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>01:11:05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.3291</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="J5" t="n">
+        <v>8300</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5850</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V5" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>0.07295218408107754</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>-0.2990956318378448</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>01:12:48</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.3291</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="J6" t="n">
+        <v>8300</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5850</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V6" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>0.07295218408107754</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>-0.2990956318378448</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>01:12:59</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.2598</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.3724</v>
+      </c>
+      <c r="J7" t="n">
+        <v>8100</v>
+      </c>
+      <c r="K7" t="n">
+        <v>850</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>13</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V7" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>0.1076062351465225</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>-0.2297875297069549</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>BUY WINNER FarmVille $11@0.490</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
         <is>
           <t>FarmVille</t>
         </is>
@@ -729,21 +1309,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="5" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -814,6 +1394,57 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>01:12:59</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>23.3469387755102</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0.6276062351465225</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>0.1076062351465225</v>
+      </c>
+      <c r="M2" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:18:55 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1298,6 +1298,434 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>01:14:43</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.1944</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.3397</v>
+      </c>
+      <c r="J8" t="n">
+        <v>11600</v>
+      </c>
+      <c r="K8" t="n">
+        <v>6400</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" t="n">
+        <v>18</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>4</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V8" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>-0.1644413036108016</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>01:16:17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.2906</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.3878</v>
+      </c>
+      <c r="J9" t="n">
+        <v>3400</v>
+      </c>
+      <c r="K9" t="n">
+        <v>8100</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>10</v>
+      </c>
+      <c r="O9" t="n">
+        <v>21</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>5</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V9" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>-0.2605883193016052</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>01:18:02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.2906</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.3878</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3400</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8100</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="O10" t="n">
+        <v>21</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V10" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>-0.2605883193016052</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>01:18:13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0.3569</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.4209</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6150</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8500</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>15</v>
+      </c>
+      <c r="O11" t="n">
+        <v>24</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>6</v>
+      </c>
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V11" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>-0.3268958342075348</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:23:57 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AD14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1726,6 +1726,327 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>01:20:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>4-4</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.466</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.4755</v>
+      </c>
+      <c r="J12" t="n">
+        <v>9950</v>
+      </c>
+      <c r="K12" t="n">
+        <v>3900</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>20</v>
+      </c>
+      <c r="O12" t="n">
+        <v>27</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>6</v>
+      </c>
+      <c r="R12" t="n">
+        <v>3</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V12" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X12" s="2" t="n">
+        <v>-0.03902370214462278</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>01:22:54</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.466</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.4755</v>
+      </c>
+      <c r="J13" t="n">
+        <v>9950</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3900</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>20</v>
+      </c>
+      <c r="O13" t="n">
+        <v>27</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>6</v>
+      </c>
+      <c r="R13" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V13" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X13" s="2" t="n">
+        <v>-0.03902370214462278</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>01:23:05</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.5248</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.5049</v>
+      </c>
+      <c r="J14" t="n">
+        <v>12200</v>
+      </c>
+      <c r="K14" t="n">
+        <v>9100</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>24</v>
+      </c>
+      <c r="O14" t="n">
+        <v>29</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>6</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V14" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X14" s="2" t="n">
+        <v>0.01975482225418093</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:29:02 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -82,6 +82,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD14"/>
+  <dimension ref="A1:AD21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2047,6 +2048,774 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>01:24:28</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.5248</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0.5049</v>
+      </c>
+      <c r="J15" t="n">
+        <v>12200</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9100</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>24</v>
+      </c>
+      <c r="O15" t="n">
+        <v>29</v>
+      </c>
+      <c r="P15" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" t="n">
+        <v>4</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V15" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X15" s="2" t="n">
+        <v>0.01975482225418093</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>WINNER:FarmVille@0.490x23</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>01:24:39</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.6038</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0.5444</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2750</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>29</v>
+      </c>
+      <c r="O16" t="n">
+        <v>31</v>
+      </c>
+      <c r="P16" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>6</v>
+      </c>
+      <c r="R16" t="n">
+        <v>5</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V16" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="X16" s="3" t="n">
+        <v>-0.3862244987487793</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB16" s="5" t="inlineStr">
+        <is>
+          <t>SELL WINNER FarmVille P/L:$-0.23</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>01:25:31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>7-4</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.6038</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0.5444</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2750</v>
+      </c>
+      <c r="K17" t="n">
+        <v>2700</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>29</v>
+      </c>
+      <c r="O17" t="n">
+        <v>31</v>
+      </c>
+      <c r="P17" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>6</v>
+      </c>
+      <c r="R17" t="n">
+        <v>5</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V17" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W17" s="2" t="n">
+        <v>-0.06438775062561028</v>
+      </c>
+      <c r="X17" s="3" t="n">
+        <v>-0.3862244987487793</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>01:25:42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>11</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>7-4</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.6971000000000001</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0.591</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5500</v>
+      </c>
+      <c r="K18" t="n">
+        <v>7800</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>34</v>
+      </c>
+      <c r="O18" t="n">
+        <v>33</v>
+      </c>
+      <c r="P18" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>6</v>
+      </c>
+      <c r="R18" t="n">
+        <v>6</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V18" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W18" s="3" t="n">
+        <v>-0.1110466539859772</v>
+      </c>
+      <c r="X18" s="3" t="n">
+        <v>-0.2929066920280456</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z18" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>01:26:56</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>8-4</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.6971000000000001</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0.591</v>
+      </c>
+      <c r="J19" t="n">
+        <v>5500</v>
+      </c>
+      <c r="K19" t="n">
+        <v>7800</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>34</v>
+      </c>
+      <c r="O19" t="n">
+        <v>33</v>
+      </c>
+      <c r="P19" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>6</v>
+      </c>
+      <c r="R19" t="n">
+        <v>6</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V19" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W19" s="3" t="n">
+        <v>-0.1110466539859772</v>
+      </c>
+      <c r="X19" s="3" t="n">
+        <v>-0.3229066920280457</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>01:27:06</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>8-4</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.7781</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>0.6316000000000001</v>
+      </c>
+      <c r="J20" t="n">
+        <v>7850</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1100</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>39</v>
+      </c>
+      <c r="O20" t="n">
+        <v>34</v>
+      </c>
+      <c r="P20" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>6</v>
+      </c>
+      <c r="R20" t="n">
+        <v>7</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V20" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W20" s="3" t="n">
+        <v>-0.1515553414821625</v>
+      </c>
+      <c r="X20" s="3" t="n">
+        <v>-0.241889317035675</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>01:28:19</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>13</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>8-5</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0.8637</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0.6743</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>44</v>
+      </c>
+      <c r="O21" t="n">
+        <v>37</v>
+      </c>
+      <c r="P21" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>6</v>
+      </c>
+      <c r="R21" t="n">
+        <v>8</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V21" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W21" s="3" t="n">
+        <v>-0.19432572722435</v>
+      </c>
+      <c r="X21" s="3" t="n">
+        <v>-0.1563485455513</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2058,7 +2827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2073,7 +2842,7 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2192,6 +2961,57 @@
       </c>
       <c r="M2" s="8" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>01:24:39</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>23.3469387755102</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>0.4556122493743897</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>-0.0543877506256103</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>-0.2334693877551022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
live update 01:34:04 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD21"/>
+  <dimension ref="A1:AD24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2816,6 +2816,336 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>01:29:54</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>14</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>9-5</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.7637</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0.6244</v>
+      </c>
+      <c r="J22" t="n">
+        <v>6200</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7400</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>48</v>
+      </c>
+      <c r="O22" t="n">
+        <v>40</v>
+      </c>
+      <c r="P22" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>6</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V22" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W22" s="3" t="n">
+        <v>-0.1443723261356354</v>
+      </c>
+      <c r="X22" s="3" t="n">
+        <v>-0.2562553477287293</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>01:31:27</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>15</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>10-5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.8534</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0.6692</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K23" t="n">
+        <v>3400</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>53</v>
+      </c>
+      <c r="O23" t="n">
+        <v>43</v>
+      </c>
+      <c r="P23" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>6</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V23" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W23" s="3" t="n">
+        <v>-0.1892139434814452</v>
+      </c>
+      <c r="X23" s="3" t="n">
+        <v>-0.1465721130371093</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>01:32:31</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>16</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>11-5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0.9235</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0.7043</v>
+      </c>
+      <c r="J24" t="n">
+        <v>8600</v>
+      </c>
+      <c r="K24" t="n">
+        <v>700</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>58</v>
+      </c>
+      <c r="O24" t="n">
+        <v>44</v>
+      </c>
+      <c r="P24" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>6</v>
+      </c>
+      <c r="R24" t="n">
+        <v>2</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V24" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W24" s="3" t="n">
+        <v>-0.2242562294006348</v>
+      </c>
+      <c r="X24" s="2" t="n">
+        <v>-0.07648754119873044</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z24" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:39:09 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD24"/>
+  <dimension ref="A1:AD30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3146,6 +3146,666 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>01:34:26</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>16</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>11-6</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0.9235</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0.7043</v>
+      </c>
+      <c r="J25" t="n">
+        <v>8600</v>
+      </c>
+      <c r="K25" t="n">
+        <v>700</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>58</v>
+      </c>
+      <c r="O25" t="n">
+        <v>44</v>
+      </c>
+      <c r="P25" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>2</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V25" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W25" s="3" t="n">
+        <v>-0.2242562294006348</v>
+      </c>
+      <c r="X25" s="2" t="n">
+        <v>-0.06648754119873043</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z25" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>01:34:37</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>17</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>11-6</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0.9644</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0.7247</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3600</v>
+      </c>
+      <c r="K26" t="n">
+        <v>800</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>63</v>
+      </c>
+      <c r="O26" t="n">
+        <v>46</v>
+      </c>
+      <c r="P26" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>6</v>
+      </c>
+      <c r="R26" t="n">
+        <v>3</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V26" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W26" s="3" t="n">
+        <v>-0.2353022980690004</v>
+      </c>
+      <c r="X26" s="2" t="n">
+        <v>-0.02560459613800045</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z26" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>01:36:21</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>17</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>11-7</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0.9644</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0.7247</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3600</v>
+      </c>
+      <c r="K27" t="n">
+        <v>800</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>63</v>
+      </c>
+      <c r="O27" t="n">
+        <v>46</v>
+      </c>
+      <c r="P27" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>6</v>
+      </c>
+      <c r="R27" t="n">
+        <v>3</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V27" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W27" s="3" t="n">
+        <v>-0.2353022980690004</v>
+      </c>
+      <c r="X27" s="2" t="n">
+        <v>-0.04560459613800047</v>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z27" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>01:36:32</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>11-7</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0.9263</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0.7057</v>
+      </c>
+      <c r="J28" t="n">
+        <v>5400</v>
+      </c>
+      <c r="K28" t="n">
+        <v>5100</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>67</v>
+      </c>
+      <c r="O28" t="n">
+        <v>51</v>
+      </c>
+      <c r="P28" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>7</v>
+      </c>
+      <c r="R28" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V28" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W28" s="3" t="n">
+        <v>-0.2256649851799011</v>
+      </c>
+      <c r="X28" s="3" t="n">
+        <v>-0.08367002964019774</v>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z28" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>01:37:55</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>12-7</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>0.9263</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0.7057</v>
+      </c>
+      <c r="J29" t="n">
+        <v>5400</v>
+      </c>
+      <c r="K29" t="n">
+        <v>5100</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>67</v>
+      </c>
+      <c r="O29" t="n">
+        <v>51</v>
+      </c>
+      <c r="P29" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>7</v>
+      </c>
+      <c r="R29" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U29" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V29" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W29" s="3" t="n">
+        <v>-0.2256649851799011</v>
+      </c>
+      <c r="X29" s="2" t="n">
+        <v>-0.06367002964019772</v>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z29" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>01:38:06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>19</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>12-7</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0.8747</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0.6798</v>
+      </c>
+      <c r="J30" t="n">
+        <v>6100</v>
+      </c>
+      <c r="K30" t="n">
+        <v>7550</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>70</v>
+      </c>
+      <c r="O30" t="n">
+        <v>56</v>
+      </c>
+      <c r="P30" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>7</v>
+      </c>
+      <c r="R30" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U30" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V30" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W30" s="3" t="n">
+        <v>-0.1998318254947662</v>
+      </c>
+      <c r="X30" s="3" t="n">
+        <v>-0.1153363490104675</v>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z30" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:44:11 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD30"/>
+  <dimension ref="A1:AD31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3806,6 +3806,116 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>01:39:41</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>20</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>13-7</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="J31" t="n">
+        <v>150</v>
+      </c>
+      <c r="K31" t="n">
+        <v>5150</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>75</v>
+      </c>
+      <c r="O31" t="n">
+        <v>58</v>
+      </c>
+      <c r="P31" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>7</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T31" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V31" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W31" s="2" t="n">
+        <v>0.01801178693771358</v>
+      </c>
+      <c r="X31" s="2" t="n">
+        <v>-0.06397642612457274</v>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z31" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:59:20 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,13 +448,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD31"/>
+  <dimension ref="A1:AD33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
@@ -3911,6 +3911,226 @@
         </is>
       </c>
       <c r="AD31" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>01:57:43</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0.5705</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0.7853</v>
+      </c>
+      <c r="J32" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K32" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T32" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V32" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W32" s="3" t="n">
+        <v>-0.1747402465343476</v>
+      </c>
+      <c r="X32" s="3" t="n">
+        <v>-0.4494804930686951</v>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z32" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>01:59:18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0.6804</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0.8401999999999999</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>4</v>
+      </c>
+      <c r="O33" t="n">
+        <v>5</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V33" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W33" s="3" t="n">
+        <v>-0.1198111391067505</v>
+      </c>
+      <c r="X33" s="3" t="n">
+        <v>-0.339622278213501</v>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z33" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
         <is>
           <t>FarmVille</t>
         </is>

</xml_diff>

<commit_message>
live update 02:04:26 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD33"/>
+  <dimension ref="A1:AD36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4136,6 +4136,336 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>02:01:25</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0.6804</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0.8401999999999999</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>4</v>
+      </c>
+      <c r="O34" t="n">
+        <v>5</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T34" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U34" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V34" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W34" s="3" t="n">
+        <v>-0.1198111391067505</v>
+      </c>
+      <c r="X34" s="3" t="n">
+        <v>-0.339622278213501</v>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z34" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>02:01:37</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0.7027</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0.8512999999999999</v>
+      </c>
+      <c r="J35" t="n">
+        <v>6500</v>
+      </c>
+      <c r="K35" t="n">
+        <v>10400</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>8</v>
+      </c>
+      <c r="O35" t="n">
+        <v>7</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>2</v>
+      </c>
+      <c r="R35" t="n">
+        <v>2</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T35" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U35" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V35" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W35" s="3" t="n">
+        <v>-0.1086698389053345</v>
+      </c>
+      <c r="X35" s="3" t="n">
+        <v>-0.317339677810669</v>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z35" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>02:03:43</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0.7208</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0.8604000000000001</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K36" t="n">
+        <v>11100</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>11</v>
+      </c>
+      <c r="O36" t="n">
+        <v>9</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>2</v>
+      </c>
+      <c r="R36" t="n">
+        <v>3</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T36" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U36" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V36" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W36" s="3" t="n">
+        <v>-0.09962182402610784</v>
+      </c>
+      <c r="X36" s="3" t="n">
+        <v>-0.2992436480522156</v>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z36" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:09:36 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD36"/>
+  <dimension ref="A1:AD42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -473,7 +473,7 @@
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="23" max="23"/>
     <col width="24" customWidth="1" min="24" max="24"/>
     <col width="27" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
@@ -4461,6 +4461,666 @@
         </is>
       </c>
       <c r="AD36" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>02:04:58</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0.7208</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>0.8604000000000001</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K37" t="n">
+        <v>11100</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>11</v>
+      </c>
+      <c r="O37" t="n">
+        <v>9</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>2</v>
+      </c>
+      <c r="R37" t="n">
+        <v>3</v>
+      </c>
+      <c r="S37" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T37" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U37" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V37" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W37" s="3" t="n">
+        <v>-0.09962182402610784</v>
+      </c>
+      <c r="X37" s="3" t="n">
+        <v>-0.2792436480522156</v>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z37" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>02:05:10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0.8221000000000001</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>0.9111</v>
+      </c>
+      <c r="J38" t="n">
+        <v>8300</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1400</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>16</v>
+      </c>
+      <c r="O38" t="n">
+        <v>10</v>
+      </c>
+      <c r="P38" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>2</v>
+      </c>
+      <c r="R38" t="n">
+        <v>4</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T38" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U38" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V38" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W38" s="2" t="n">
+        <v>-0.04894726634025579</v>
+      </c>
+      <c r="X38" s="3" t="n">
+        <v>-0.1778945326805114</v>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z38" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>02:06:34</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0.8221000000000001</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>0.9111</v>
+      </c>
+      <c r="J39" t="n">
+        <v>8300</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1400</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>16</v>
+      </c>
+      <c r="O39" t="n">
+        <v>10</v>
+      </c>
+      <c r="P39" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>2</v>
+      </c>
+      <c r="R39" t="n">
+        <v>4</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U39" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V39" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W39" s="2" t="n">
+        <v>-0.04894726634025579</v>
+      </c>
+      <c r="X39" s="3" t="n">
+        <v>-0.1678945326805114</v>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z39" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>02:06:45</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0.7376</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="J40" t="n">
+        <v>6500</v>
+      </c>
+      <c r="K40" t="n">
+        <v>4150</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>20</v>
+      </c>
+      <c r="O40" t="n">
+        <v>15</v>
+      </c>
+      <c r="P40" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>2</v>
+      </c>
+      <c r="R40" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T40" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U40" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V40" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W40" s="3" t="n">
+        <v>-0.09118323683738713</v>
+      </c>
+      <c r="X40" s="3" t="n">
+        <v>-0.2523664736747742</v>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z40" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>02:07:39</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>6</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>0.7376</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>0.8688</v>
+      </c>
+      <c r="J41" t="n">
+        <v>6500</v>
+      </c>
+      <c r="K41" t="n">
+        <v>4150</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>20</v>
+      </c>
+      <c r="O41" t="n">
+        <v>15</v>
+      </c>
+      <c r="P41" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2</v>
+      </c>
+      <c r="R41" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S41" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T41" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U41" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V41" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W41" s="3" t="n">
+        <v>-0.09118323683738713</v>
+      </c>
+      <c r="X41" s="3" t="n">
+        <v>-0.2723664736747742</v>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z41" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>02:07:50</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>7</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="J42" t="n">
+        <v>6100</v>
+      </c>
+      <c r="K42" t="n">
+        <v>7200</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>21</v>
+      </c>
+      <c r="O42" t="n">
+        <v>20</v>
+      </c>
+      <c r="P42" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>3</v>
+      </c>
+      <c r="R42" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T42" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U42" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V42" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W42" s="3" t="n">
+        <v>-0.1425159788131714</v>
+      </c>
+      <c r="X42" s="3" t="n">
+        <v>-0.3750319576263428</v>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z42" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
         <is>
           <t>FarmVille</t>
         </is>

</xml_diff>

<commit_message>
live update 02:14:44 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD42"/>
+  <dimension ref="A1:AD48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5126,6 +5126,666 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>02:10:28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>7</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>4-4</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="J43" t="n">
+        <v>6100</v>
+      </c>
+      <c r="K43" t="n">
+        <v>7200</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>21</v>
+      </c>
+      <c r="O43" t="n">
+        <v>20</v>
+      </c>
+      <c r="P43" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>3</v>
+      </c>
+      <c r="R43" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S43" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T43" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U43" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V43" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W43" s="3" t="n">
+        <v>-0.1425159788131714</v>
+      </c>
+      <c r="X43" s="3" t="n">
+        <v>-0.3550319576263428</v>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z43" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>02:10:40</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>8</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>4-4</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>0.579</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>0.7895</v>
+      </c>
+      <c r="J44" t="n">
+        <v>8100</v>
+      </c>
+      <c r="K44" t="n">
+        <v>9750</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>21</v>
+      </c>
+      <c r="O44" t="n">
+        <v>25</v>
+      </c>
+      <c r="P44" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>4</v>
+      </c>
+      <c r="R44" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T44" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U44" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V44" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W44" s="3" t="n">
+        <v>-0.1704896306991578</v>
+      </c>
+      <c r="X44" s="3" t="n">
+        <v>-0.4109792613983154</v>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z44" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>02:12:14</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>8</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>0.579</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>0.7895</v>
+      </c>
+      <c r="J45" t="n">
+        <v>8100</v>
+      </c>
+      <c r="K45" t="n">
+        <v>9750</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>21</v>
+      </c>
+      <c r="O45" t="n">
+        <v>25</v>
+      </c>
+      <c r="P45" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>4</v>
+      </c>
+      <c r="R45" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S45" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T45" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U45" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V45" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W45" s="3" t="n">
+        <v>-0.1704896306991578</v>
+      </c>
+      <c r="X45" s="3" t="n">
+        <v>-0.4309792613983154</v>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z45" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>02:12:26</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>9</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0.4482</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>0.7241</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K46" t="n">
+        <v>11900</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>24</v>
+      </c>
+      <c r="O46" t="n">
+        <v>30</v>
+      </c>
+      <c r="P46" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>5</v>
+      </c>
+      <c r="R46" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T46" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U46" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V46" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W46" s="3" t="n">
+        <v>-0.2359049087762833</v>
+      </c>
+      <c r="X46" s="2" t="n">
+        <v>-0.07180981755256652</v>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z46" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>02:14:01</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>9</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0.4482</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>0.7241</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K47" t="n">
+        <v>11900</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>24</v>
+      </c>
+      <c r="O47" t="n">
+        <v>30</v>
+      </c>
+      <c r="P47" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>5</v>
+      </c>
+      <c r="R47" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S47" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T47" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U47" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V47" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W47" s="3" t="n">
+        <v>-0.2359049087762833</v>
+      </c>
+      <c r="X47" s="2" t="n">
+        <v>-0.07180981755256652</v>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z47" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>02:14:12</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>10</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0.4606</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>0.7302999999999999</v>
+      </c>
+      <c r="J48" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2650</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>28</v>
+      </c>
+      <c r="O48" t="n">
+        <v>35</v>
+      </c>
+      <c r="P48" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>5</v>
+      </c>
+      <c r="R48" t="n">
+        <v>-5</v>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T48" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U48" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V48" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W48" s="3" t="n">
+        <v>-0.2296956843137742</v>
+      </c>
+      <c r="X48" s="2" t="n">
+        <v>-0.05939136862754821</v>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z48" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:19:51 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD48"/>
+  <dimension ref="A1:AD52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5786,6 +5786,446 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>02:15:58</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>10</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>0.4606</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>0.7302999999999999</v>
+      </c>
+      <c r="J49" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K49" t="n">
+        <v>2650</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>28</v>
+      </c>
+      <c r="O49" t="n">
+        <v>35</v>
+      </c>
+      <c r="P49" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>5</v>
+      </c>
+      <c r="R49" t="n">
+        <v>-5</v>
+      </c>
+      <c r="S49" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T49" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U49" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V49" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W49" s="3" t="n">
+        <v>-0.2296956843137742</v>
+      </c>
+      <c r="X49" s="2" t="n">
+        <v>-0.05939136862754821</v>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z49" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>02:16:09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>11</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0.4267</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0.7133</v>
+      </c>
+      <c r="J50" t="n">
+        <v>600</v>
+      </c>
+      <c r="K50" t="n">
+        <v>5200</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>29</v>
+      </c>
+      <c r="O50" t="n">
+        <v>40</v>
+      </c>
+      <c r="P50" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>6</v>
+      </c>
+      <c r="R50" t="n">
+        <v>-6</v>
+      </c>
+      <c r="S50" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T50" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U50" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V50" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W50" s="3" t="n">
+        <v>-0.2333423686027527</v>
+      </c>
+      <c r="X50" s="3" t="n">
+        <v>-0.3966847372055053</v>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z50" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>02:17:54</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>11</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>6-6</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0.4267</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>0.7133</v>
+      </c>
+      <c r="J51" t="n">
+        <v>600</v>
+      </c>
+      <c r="K51" t="n">
+        <v>5200</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>29</v>
+      </c>
+      <c r="O51" t="n">
+        <v>40</v>
+      </c>
+      <c r="P51" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>6</v>
+      </c>
+      <c r="R51" t="n">
+        <v>-6</v>
+      </c>
+      <c r="S51" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T51" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U51" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V51" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W51" s="3" t="n">
+        <v>-0.2333423686027527</v>
+      </c>
+      <c r="X51" s="3" t="n">
+        <v>-0.3966847372055053</v>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z51" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>02:18:06</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>12</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>6-6</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>0.5377999999999999</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>0.7689</v>
+      </c>
+      <c r="J52" t="n">
+        <v>7100</v>
+      </c>
+      <c r="K52" t="n">
+        <v>900</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>34</v>
+      </c>
+      <c r="O52" t="n">
+        <v>44</v>
+      </c>
+      <c r="P52" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>7</v>
+      </c>
+      <c r="R52" t="n">
+        <v>1</v>
+      </c>
+      <c r="S52" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T52" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U52" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V52" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W52" s="3" t="n">
+        <v>-0.1911054766178132</v>
+      </c>
+      <c r="X52" s="2" t="n">
+        <v>0.01778904676437379</v>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z52" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:24:59 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD52"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6226,6 +6226,446 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>02:20:02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>13</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>6-7</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>0.6352</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="J53" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K53" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>39</v>
+      </c>
+      <c r="O53" t="n">
+        <v>47</v>
+      </c>
+      <c r="P53" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>8</v>
+      </c>
+      <c r="R53" t="n">
+        <v>2</v>
+      </c>
+      <c r="S53" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T53" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U53" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V53" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W53" s="3" t="n">
+        <v>-0.1424189722537995</v>
+      </c>
+      <c r="X53" s="3" t="n">
+        <v>-0.3648379445075989</v>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z53" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>02:21:48</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>13</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0.6352</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>0.8176</v>
+      </c>
+      <c r="J54" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K54" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>39</v>
+      </c>
+      <c r="O54" t="n">
+        <v>47</v>
+      </c>
+      <c r="P54" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>8</v>
+      </c>
+      <c r="R54" t="n">
+        <v>2</v>
+      </c>
+      <c r="S54" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T54" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U54" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V54" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W54" s="3" t="n">
+        <v>-0.1424189722537995</v>
+      </c>
+      <c r="X54" s="3" t="n">
+        <v>-0.3848379445075989</v>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z54" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>02:22:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>14</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0.5088</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0.7544</v>
+      </c>
+      <c r="J55" t="n">
+        <v>11600</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>41</v>
+      </c>
+      <c r="O55" t="n">
+        <v>52</v>
+      </c>
+      <c r="P55" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>8</v>
+      </c>
+      <c r="R55" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S55" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T55" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U55" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V55" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W55" s="3" t="n">
+        <v>-0.2056136941909791</v>
+      </c>
+      <c r="X55" s="2" t="n">
+        <v>-0.011227388381958</v>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z55" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>02:23:34</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>15</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>6-9</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0.4493</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0.7246</v>
+      </c>
+      <c r="J56" t="n">
+        <v>9800</v>
+      </c>
+      <c r="K56" t="n">
+        <v>7100</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>44</v>
+      </c>
+      <c r="O56" t="n">
+        <v>57</v>
+      </c>
+      <c r="P56" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>8</v>
+      </c>
+      <c r="R56" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S56" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T56" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U56" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V56" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W56" s="3" t="n">
+        <v>-0.2353625810146332</v>
+      </c>
+      <c r="X56" s="2" t="n">
+        <v>-0.07072516202926635</v>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z56" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:30:06 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A1:AD59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6666,6 +6666,336 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>02:26:33</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>16</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>7-9</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>0.3412</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>0.6706</v>
+      </c>
+      <c r="J57" t="n">
+        <v>10200</v>
+      </c>
+      <c r="K57" t="n">
+        <v>2400</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>47</v>
+      </c>
+      <c r="O57" t="n">
+        <v>62</v>
+      </c>
+      <c r="P57" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>9</v>
+      </c>
+      <c r="R57" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S57" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T57" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U57" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V57" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W57" s="3" t="n">
+        <v>-0.190582965016365</v>
+      </c>
+      <c r="X57" s="3" t="n">
+        <v>-0.3111659300327301</v>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z57" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>02:29:01</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>16</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>7-10</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>0.3412</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>0.6706</v>
+      </c>
+      <c r="J58" t="n">
+        <v>10200</v>
+      </c>
+      <c r="K58" t="n">
+        <v>2400</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>47</v>
+      </c>
+      <c r="O58" t="n">
+        <v>62</v>
+      </c>
+      <c r="P58" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>9</v>
+      </c>
+      <c r="R58" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S58" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T58" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U58" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V58" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W58" s="3" t="n">
+        <v>-0.190582965016365</v>
+      </c>
+      <c r="X58" s="3" t="n">
+        <v>-0.3111659300327301</v>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z58" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>02:29:12</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>17</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>7-10</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>0.5159</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="J59" t="n">
+        <v>12450</v>
+      </c>
+      <c r="K59" t="n">
+        <v>9500</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>51</v>
+      </c>
+      <c r="O59" t="n">
+        <v>63</v>
+      </c>
+      <c r="P59" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>9</v>
+      </c>
+      <c r="R59" t="n">
+        <v>1</v>
+      </c>
+      <c r="S59" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T59" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U59" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V59" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W59" s="3" t="n">
+        <v>-0.2020307993888855</v>
+      </c>
+      <c r="X59" s="2" t="n">
+        <v>-0.004061598777770986</v>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z59" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:35:14 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD59"/>
+  <dimension ref="A1:AD63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6996,6 +6996,446 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>02:31:51</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>17</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>7-11</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0.5159</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="J60" t="n">
+        <v>12450</v>
+      </c>
+      <c r="K60" t="n">
+        <v>9500</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>51</v>
+      </c>
+      <c r="O60" t="n">
+        <v>63</v>
+      </c>
+      <c r="P60" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>9</v>
+      </c>
+      <c r="R60" t="n">
+        <v>1</v>
+      </c>
+      <c r="S60" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T60" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U60" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V60" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W60" s="3" t="n">
+        <v>-0.2020307993888855</v>
+      </c>
+      <c r="X60" s="2" t="n">
+        <v>-0.004061598777770986</v>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z60" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>02:32:02</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>18</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>7-11</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>0.3076</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>0.6538</v>
+      </c>
+      <c r="J61" t="n">
+        <v>850</v>
+      </c>
+      <c r="K61" t="n">
+        <v>4400</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>54</v>
+      </c>
+      <c r="O61" t="n">
+        <v>68</v>
+      </c>
+      <c r="P61" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>10</v>
+      </c>
+      <c r="R61" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S61" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T61" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U61" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V61" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W61" s="3" t="n">
+        <v>-0.1737871658802032</v>
+      </c>
+      <c r="X61" s="3" t="n">
+        <v>-0.2775743317604065</v>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z61" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>02:34:18</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>18</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0.3076</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>0.6538</v>
+      </c>
+      <c r="J62" t="n">
+        <v>850</v>
+      </c>
+      <c r="K62" t="n">
+        <v>4400</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>54</v>
+      </c>
+      <c r="O62" t="n">
+        <v>68</v>
+      </c>
+      <c r="P62" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>10</v>
+      </c>
+      <c r="R62" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S62" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T62" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U62" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V62" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W62" s="3" t="n">
+        <v>-0.1737871658802032</v>
+      </c>
+      <c r="X62" s="3" t="n">
+        <v>-0.2775743317604065</v>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z62" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>02:34:30</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>19</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>0.1714</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>0.5857</v>
+      </c>
+      <c r="J63" t="n">
+        <v>3750</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>56</v>
+      </c>
+      <c r="O63" t="n">
+        <v>72</v>
+      </c>
+      <c r="P63" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>11</v>
+      </c>
+      <c r="R63" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S63" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T63" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U63" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V63" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W63" s="3" t="n">
+        <v>-0.1057111513614654</v>
+      </c>
+      <c r="X63" s="3" t="n">
+        <v>-0.1414223027229309</v>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z63" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:40:22 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD63"/>
+  <dimension ref="A1:AD67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7436,6 +7436,446 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>02:36:16</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>19</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>9-11</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>0.1714</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>0.5857</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3750</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>56</v>
+      </c>
+      <c r="O64" t="n">
+        <v>72</v>
+      </c>
+      <c r="P64" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>11</v>
+      </c>
+      <c r="R64" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S64" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T64" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U64" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V64" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W64" s="3" t="n">
+        <v>-0.1057111513614654</v>
+      </c>
+      <c r="X64" s="3" t="n">
+        <v>-0.1414223027229309</v>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z64" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>02:36:28</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>20</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>9-11</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>0.3163</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0.6582</v>
+      </c>
+      <c r="J65" t="n">
+        <v>6100</v>
+      </c>
+      <c r="K65" t="n">
+        <v>7400</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>61</v>
+      </c>
+      <c r="O65" t="n">
+        <v>74</v>
+      </c>
+      <c r="P65" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>11</v>
+      </c>
+      <c r="R65" t="n">
+        <v>1</v>
+      </c>
+      <c r="S65" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T65" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U65" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V65" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W65" s="3" t="n">
+        <v>-0.17815469622612</v>
+      </c>
+      <c r="X65" s="3" t="n">
+        <v>-0.28630939245224</v>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z65" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>02:38:55</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>20</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>0.3163</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0.6582</v>
+      </c>
+      <c r="J66" t="n">
+        <v>6100</v>
+      </c>
+      <c r="K66" t="n">
+        <v>7400</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>61</v>
+      </c>
+      <c r="O66" t="n">
+        <v>74</v>
+      </c>
+      <c r="P66" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>11</v>
+      </c>
+      <c r="R66" t="n">
+        <v>1</v>
+      </c>
+      <c r="S66" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T66" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U66" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V66" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W66" s="3" t="n">
+        <v>-0.17815469622612</v>
+      </c>
+      <c r="X66" s="3" t="n">
+        <v>-0.28630939245224</v>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z66" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>02:39:07</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>21</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>0.4328</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>0.7164</v>
+      </c>
+      <c r="J67" t="n">
+        <v>8450</v>
+      </c>
+      <c r="K67" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>66</v>
+      </c>
+      <c r="O67" t="n">
+        <v>75</v>
+      </c>
+      <c r="P67" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>11</v>
+      </c>
+      <c r="R67" t="n">
+        <v>2</v>
+      </c>
+      <c r="S67" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T67" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U67" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V67" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W67" s="3" t="n">
+        <v>-0.2364060920476913</v>
+      </c>
+      <c r="X67" s="3" t="n">
+        <v>-0.4028121840953827</v>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z67" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:45:22 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD67"/>
+  <dimension ref="A1:AD73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7876,6 +7876,666 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>02:41:35</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>21</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0.4328</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0.7164</v>
+      </c>
+      <c r="J68" t="n">
+        <v>8450</v>
+      </c>
+      <c r="K68" t="n">
+        <v>7500</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>66</v>
+      </c>
+      <c r="O68" t="n">
+        <v>75</v>
+      </c>
+      <c r="P68" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>11</v>
+      </c>
+      <c r="R68" t="n">
+        <v>2</v>
+      </c>
+      <c r="S68" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T68" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U68" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V68" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W68" s="3" t="n">
+        <v>-0.2364060920476913</v>
+      </c>
+      <c r="X68" s="3" t="n">
+        <v>-0.4028121840953827</v>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z68" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB68" t="inlineStr"/>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>02:41:47</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>22</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="n">
+        <v>0.1245</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>0.5623</v>
+      </c>
+      <c r="J69" t="n">
+        <v>8350</v>
+      </c>
+      <c r="K69" t="n">
+        <v>2800</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>68</v>
+      </c>
+      <c r="O69" t="n">
+        <v>80</v>
+      </c>
+      <c r="P69" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>11</v>
+      </c>
+      <c r="R69" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S69" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T69" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U69" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V69" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W69" s="3" t="n">
+        <v>-0.08225135549902915</v>
+      </c>
+      <c r="X69" s="3" t="n">
+        <v>-0.09450271099805826</v>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z69" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>02:42:40</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>22</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>11-12</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>0.1245</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>0.5623</v>
+      </c>
+      <c r="J70" t="n">
+        <v>8350</v>
+      </c>
+      <c r="K70" t="n">
+        <v>2800</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>68</v>
+      </c>
+      <c r="O70" t="n">
+        <v>80</v>
+      </c>
+      <c r="P70" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>11</v>
+      </c>
+      <c r="R70" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S70" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T70" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U70" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V70" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W70" s="3" t="n">
+        <v>-0.08225135549902915</v>
+      </c>
+      <c r="X70" s="3" t="n">
+        <v>-0.09450271099805826</v>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z70" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>02:42:52</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>23</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>11-12</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>0.6331</v>
+      </c>
+      <c r="J71" t="n">
+        <v>12150</v>
+      </c>
+      <c r="K71" t="n">
+        <v>7100</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>73</v>
+      </c>
+      <c r="O71" t="n">
+        <v>84</v>
+      </c>
+      <c r="P71" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>12</v>
+      </c>
+      <c r="R71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S71" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T71" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U71" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V71" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W71" s="3" t="n">
+        <v>-0.1531142038106918</v>
+      </c>
+      <c r="X71" s="3" t="n">
+        <v>-0.2362284076213836</v>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z71" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>02:44:37</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>23</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>12-12</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>0.6331</v>
+      </c>
+      <c r="J72" t="n">
+        <v>12150</v>
+      </c>
+      <c r="K72" t="n">
+        <v>7100</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>73</v>
+      </c>
+      <c r="O72" t="n">
+        <v>84</v>
+      </c>
+      <c r="P72" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>12</v>
+      </c>
+      <c r="R72" t="n">
+        <v>1</v>
+      </c>
+      <c r="S72" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T72" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U72" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V72" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W72" s="3" t="n">
+        <v>-0.1531142038106918</v>
+      </c>
+      <c r="X72" s="3" t="n">
+        <v>-0.2362284076213836</v>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z72" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>02:44:49</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>24</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>12-12</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>0.3364</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>0.6682</v>
+      </c>
+      <c r="J73" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K73" t="n">
+        <v>9100</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>78</v>
+      </c>
+      <c r="O73" t="n">
+        <v>84</v>
+      </c>
+      <c r="P73" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>12</v>
+      </c>
+      <c r="R73" t="n">
+        <v>2</v>
+      </c>
+      <c r="S73" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T73" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U73" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V73" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W73" s="3" t="n">
+        <v>-0.1882246476411819</v>
+      </c>
+      <c r="X73" s="3" t="n">
+        <v>-0.3064492952823639</v>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z73" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:50:22 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD73"/>
+  <dimension ref="A1:AD79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8536,6 +8536,666 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>02:46:15</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>24</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>12-13</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0.3364</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>0.6682</v>
+      </c>
+      <c r="J74" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K74" t="n">
+        <v>9100</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>78</v>
+      </c>
+      <c r="O74" t="n">
+        <v>84</v>
+      </c>
+      <c r="P74" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>12</v>
+      </c>
+      <c r="R74" t="n">
+        <v>2</v>
+      </c>
+      <c r="S74" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T74" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U74" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V74" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W74" s="3" t="n">
+        <v>-0.1882246476411819</v>
+      </c>
+      <c r="X74" s="3" t="n">
+        <v>-0.3064492952823639</v>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z74" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>02:46:26</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>25</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>12-13</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>0.6163999999999999</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>0.8082</v>
+      </c>
+      <c r="J75" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K75" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>83</v>
+      </c>
+      <c r="O75" t="n">
+        <v>86</v>
+      </c>
+      <c r="P75" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>13</v>
+      </c>
+      <c r="R75" t="n">
+        <v>3</v>
+      </c>
+      <c r="S75" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T75" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U75" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V75" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W75" s="3" t="n">
+        <v>-0.1518205916881562</v>
+      </c>
+      <c r="X75" s="3" t="n">
+        <v>-0.3736411833763122</v>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z75" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>02:47:20</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>25</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>13-13</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0.6163999999999999</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>0.8082</v>
+      </c>
+      <c r="J76" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K76" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>83</v>
+      </c>
+      <c r="O76" t="n">
+        <v>86</v>
+      </c>
+      <c r="P76" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>13</v>
+      </c>
+      <c r="R76" t="n">
+        <v>3</v>
+      </c>
+      <c r="S76" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T76" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U76" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V76" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W76" s="3" t="n">
+        <v>-0.1518205916881562</v>
+      </c>
+      <c r="X76" s="3" t="n">
+        <v>-0.4036411833763123</v>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z76" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>02:47:32</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>26</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>13-13</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>0.3722</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>0.6861</v>
+      </c>
+      <c r="J77" t="n">
+        <v>33100</v>
+      </c>
+      <c r="K77" t="n">
+        <v>44800</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
+        <v>85</v>
+      </c>
+      <c r="O77" t="n">
+        <v>91</v>
+      </c>
+      <c r="P77" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>14</v>
+      </c>
+      <c r="R77" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S77" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T77" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U77" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V77" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W77" s="3" t="n">
+        <v>-0.2061198246479034</v>
+      </c>
+      <c r="X77" s="3" t="n">
+        <v>-0.3422396492958069</v>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z77" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB77" t="inlineStr"/>
+      <c r="AC77" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>02:49:38</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>26</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>13-14</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>0.3722</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>0.6861</v>
+      </c>
+      <c r="J78" t="n">
+        <v>33100</v>
+      </c>
+      <c r="K78" t="n">
+        <v>44800</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>85</v>
+      </c>
+      <c r="O78" t="n">
+        <v>91</v>
+      </c>
+      <c r="P78" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>14</v>
+      </c>
+      <c r="R78" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S78" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T78" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U78" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V78" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W78" s="3" t="n">
+        <v>-0.2061198246479034</v>
+      </c>
+      <c r="X78" s="3" t="n">
+        <v>-0.3422396492958069</v>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z78" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>02:49:49</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>27</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>13-14</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>0.6498</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>0.8249</v>
+      </c>
+      <c r="J79" t="n">
+        <v>23450</v>
+      </c>
+      <c r="K79" t="n">
+        <v>30300</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
+        <v>90</v>
+      </c>
+      <c r="O79" t="n">
+        <v>91</v>
+      </c>
+      <c r="P79" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>14</v>
+      </c>
+      <c r="R79" t="n">
+        <v>1</v>
+      </c>
+      <c r="S79" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T79" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U79" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V79" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W79" s="3" t="n">
+        <v>-0.1351128137111664</v>
+      </c>
+      <c r="X79" s="3" t="n">
+        <v>-0.3702256274223328</v>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z79" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB79" t="inlineStr"/>
+      <c r="AC79" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 02:55:29 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD79"/>
+  <dimension ref="A1:AD81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9196,6 +9196,226 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>02:51:57</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>27</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>14-14</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>0.6498</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>0.8249</v>
+      </c>
+      <c r="J80" t="n">
+        <v>23450</v>
+      </c>
+      <c r="K80" t="n">
+        <v>30300</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>90</v>
+      </c>
+      <c r="O80" t="n">
+        <v>91</v>
+      </c>
+      <c r="P80" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>14</v>
+      </c>
+      <c r="R80" t="n">
+        <v>1</v>
+      </c>
+      <c r="S80" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T80" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U80" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V80" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W80" s="3" t="n">
+        <v>-0.1351128137111664</v>
+      </c>
+      <c r="X80" s="3" t="n">
+        <v>-0.3702256274223328</v>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z80" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>02:52:09</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>28</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>14-14</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>0.2834</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>0.6417</v>
+      </c>
+      <c r="J81" t="n">
+        <v>6850</v>
+      </c>
+      <c r="K81" t="n">
+        <v>25300</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
+        <v>93</v>
+      </c>
+      <c r="O81" t="n">
+        <v>96</v>
+      </c>
+      <c r="P81" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>14</v>
+      </c>
+      <c r="R81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S81" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T81" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U81" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V81" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W81" s="3" t="n">
+        <v>-0.1617165100574493</v>
+      </c>
+      <c r="X81" s="3" t="n">
+        <v>-0.2534330201148987</v>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z81" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 03:00:37 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD81"/>
+  <dimension ref="A1:AD86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9416,6 +9416,556 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>02:55:39</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>28</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>15-14</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>0.2834</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>0.6417</v>
+      </c>
+      <c r="J82" t="n">
+        <v>6850</v>
+      </c>
+      <c r="K82" t="n">
+        <v>25300</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>93</v>
+      </c>
+      <c r="O82" t="n">
+        <v>96</v>
+      </c>
+      <c r="P82" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>14</v>
+      </c>
+      <c r="R82" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S82" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T82" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U82" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V82" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W82" s="3" t="n">
+        <v>-0.1617165100574493</v>
+      </c>
+      <c r="X82" s="3" t="n">
+        <v>-0.2534330201148987</v>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z82" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB82" t="inlineStr"/>
+      <c r="AC82" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>02:55:51</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>2</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>29</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>15-14</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>0.4731</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>0.7365</v>
+      </c>
+      <c r="J83" t="n">
+        <v>1650</v>
+      </c>
+      <c r="K83" t="n">
+        <v>8400</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>98</v>
+      </c>
+      <c r="O83" t="n">
+        <v>98</v>
+      </c>
+      <c r="P83" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>14</v>
+      </c>
+      <c r="R83" t="n">
+        <v>1</v>
+      </c>
+      <c r="S83" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T83" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U83" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V83" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W83" s="3" t="n">
+        <v>-0.2234669691324234</v>
+      </c>
+      <c r="X83" s="2" t="n">
+        <v>-0.04693393826484679</v>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z83" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB83" t="inlineStr"/>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>02:58:38</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>29</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>15-15</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>0.4731</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>0.7365</v>
+      </c>
+      <c r="J84" t="n">
+        <v>1650</v>
+      </c>
+      <c r="K84" t="n">
+        <v>8400</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>98</v>
+      </c>
+      <c r="O84" t="n">
+        <v>98</v>
+      </c>
+      <c r="P84" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>14</v>
+      </c>
+      <c r="R84" t="n">
+        <v>1</v>
+      </c>
+      <c r="S84" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T84" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U84" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V84" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W84" s="3" t="n">
+        <v>-0.2234669691324234</v>
+      </c>
+      <c r="X84" s="2" t="n">
+        <v>-0.04693393826484679</v>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z84" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB84" t="inlineStr"/>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>02:58:49</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>30</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>15-15</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>0.8295</v>
+      </c>
+      <c r="J85" t="n">
+        <v>7950</v>
+      </c>
+      <c r="K85" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>103</v>
+      </c>
+      <c r="O85" t="n">
+        <v>100</v>
+      </c>
+      <c r="P85" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>14</v>
+      </c>
+      <c r="R85" t="n">
+        <v>2</v>
+      </c>
+      <c r="S85" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T85" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U85" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V85" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W85" s="3" t="n">
+        <v>-0.1304870760440827</v>
+      </c>
+      <c r="X85" s="3" t="n">
+        <v>-0.3309741520881653</v>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z85" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB85" t="inlineStr"/>
+      <c r="AC85" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>03:00:35</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>30</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>15-16</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>0.8295</v>
+      </c>
+      <c r="J86" t="n">
+        <v>7950</v>
+      </c>
+      <c r="K86" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>103</v>
+      </c>
+      <c r="O86" t="n">
+        <v>100</v>
+      </c>
+      <c r="P86" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>14</v>
+      </c>
+      <c r="R86" t="n">
+        <v>2</v>
+      </c>
+      <c r="S86" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T86" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U86" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V86" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W86" s="3" t="n">
+        <v>-0.1304870760440827</v>
+      </c>
+      <c r="X86" s="3" t="n">
+        <v>-0.3509741520881653</v>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z86" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB86" t="inlineStr"/>
+      <c r="AC86" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 03:05:46 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD86"/>
+  <dimension ref="A1:AD91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9966,6 +9966,556 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>03:00:48</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>31</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>15-16</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>0.5262</v>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>0.7631</v>
+      </c>
+      <c r="J87" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K87" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N87" t="n">
+        <v>106</v>
+      </c>
+      <c r="O87" t="n">
+        <v>104</v>
+      </c>
+      <c r="P87" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>15</v>
+      </c>
+      <c r="R87" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S87" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T87" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U87" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V87" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W87" s="3" t="n">
+        <v>-0.1968831932544709</v>
+      </c>
+      <c r="X87" s="2" t="n">
+        <v>0.00623361349105836</v>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z87" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB87" t="inlineStr"/>
+      <c r="AC87" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>03:03:25</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>31</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>16-16</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>0.5262</v>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>0.7631</v>
+      </c>
+      <c r="J88" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K88" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>106</v>
+      </c>
+      <c r="O88" t="n">
+        <v>104</v>
+      </c>
+      <c r="P88" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>15</v>
+      </c>
+      <c r="R88" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S88" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T88" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U88" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V88" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W88" s="3" t="n">
+        <v>-0.1968831932544709</v>
+      </c>
+      <c r="X88" s="2" t="n">
+        <v>0.00623361349105836</v>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z88" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB88" t="inlineStr"/>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>03:03:37</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>32</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>16-16</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>0.2626</v>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>0.6313</v>
+      </c>
+      <c r="J89" t="n">
+        <v>36100</v>
+      </c>
+      <c r="K89" t="n">
+        <v>40350</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N89" t="n">
+        <v>108</v>
+      </c>
+      <c r="O89" t="n">
+        <v>109</v>
+      </c>
+      <c r="P89" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>15</v>
+      </c>
+      <c r="R89" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S89" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T89" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U89" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V89" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W89" s="3" t="n">
+        <v>-0.1513094943761825</v>
+      </c>
+      <c r="X89" s="3" t="n">
+        <v>-0.2326189887523651</v>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z89" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB89" t="inlineStr"/>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>03:05:12</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>32</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>17-16</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>0.2626</v>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>0.6313</v>
+      </c>
+      <c r="J90" t="n">
+        <v>36100</v>
+      </c>
+      <c r="K90" t="n">
+        <v>40350</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>108</v>
+      </c>
+      <c r="O90" t="n">
+        <v>109</v>
+      </c>
+      <c r="P90" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>15</v>
+      </c>
+      <c r="R90" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S90" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T90" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U90" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V90" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W90" s="3" t="n">
+        <v>-0.1513094943761825</v>
+      </c>
+      <c r="X90" s="3" t="n">
+        <v>-0.2326189887523651</v>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z90" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB90" t="inlineStr"/>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>03:05:24</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>33</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>17-16</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>0.5092</v>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>0.7546</v>
+      </c>
+      <c r="J91" t="n">
+        <v>30900</v>
+      </c>
+      <c r="K91" t="n">
+        <v>23750</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>113</v>
+      </c>
+      <c r="O91" t="n">
+        <v>112</v>
+      </c>
+      <c r="P91" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>15</v>
+      </c>
+      <c r="R91" t="n">
+        <v>1</v>
+      </c>
+      <c r="S91" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T91" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U91" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V91" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W91" s="3" t="n">
+        <v>-0.205417058467865</v>
+      </c>
+      <c r="X91" s="2" t="n">
+        <v>-0.01083411693572997</v>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z91" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB91" t="inlineStr"/>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 03:10:23 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-farmvi-akimbo-2026-04-02_20260403_001542.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD91"/>
+  <dimension ref="A1:AD94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10516,6 +10516,336 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>03:07:00</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>34</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>18-16</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="n">
+        <v>0.7225</v>
+      </c>
+      <c r="I92" s="2" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="J92" t="n">
+        <v>25700</v>
+      </c>
+      <c r="K92" t="n">
+        <v>8750</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>118</v>
+      </c>
+      <c r="O92" t="n">
+        <v>112</v>
+      </c>
+      <c r="P92" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>15</v>
+      </c>
+      <c r="R92" t="n">
+        <v>2</v>
+      </c>
+      <c r="S92" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T92" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U92" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V92" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W92" s="3" t="n">
+        <v>-0.09875398039817815</v>
+      </c>
+      <c r="X92" s="3" t="n">
+        <v>-0.2975079607963562</v>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z92" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB92" t="inlineStr"/>
+      <c r="AC92" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>03:08:56</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>34</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>18-17</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>0.7225</v>
+      </c>
+      <c r="I93" s="2" t="n">
+        <v>0.8612</v>
+      </c>
+      <c r="J93" t="n">
+        <v>25700</v>
+      </c>
+      <c r="K93" t="n">
+        <v>8750</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>118</v>
+      </c>
+      <c r="O93" t="n">
+        <v>112</v>
+      </c>
+      <c r="P93" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>15</v>
+      </c>
+      <c r="R93" t="n">
+        <v>2</v>
+      </c>
+      <c r="S93" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T93" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U93" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V93" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W93" s="3" t="n">
+        <v>-0.09875398039817815</v>
+      </c>
+      <c r="X93" s="3" t="n">
+        <v>-0.2975079607963562</v>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z93" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB93" t="inlineStr"/>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>03:09:08</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>overpass</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>35</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>18-17</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>0.8935999999999999</v>
+      </c>
+      <c r="I94" s="2" t="n">
+        <v>0.9468</v>
+      </c>
+      <c r="J94" t="n">
+        <v>16050</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>123</v>
+      </c>
+      <c r="O94" t="n">
+        <v>113</v>
+      </c>
+      <c r="P94" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>15</v>
+      </c>
+      <c r="R94" t="n">
+        <v>3</v>
+      </c>
+      <c r="S94" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="T94" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="U94" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="V94" t="n">
+        <v>38.123</v>
+      </c>
+      <c r="W94" s="2" t="n">
+        <v>-0.01318737030029302</v>
+      </c>
+      <c r="X94" s="3" t="n">
+        <v>-0.1263747406005859</v>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z94" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AA94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB94" t="inlineStr"/>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>F5 Esports</t>
+        </is>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>FarmVille</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>